<commit_message>
Update audit_data.xlsx from Google Sheets
</commit_message>
<xml_diff>
--- a/audit_data.xlsx
+++ b/audit_data.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:FQ13"/>
+  <dimension ref="A1:FQ12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1889,12 +1889,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>ASFGF</t>
+          <t>RGSDG</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>ASFCdE</t>
+          <t>DZSVBZDV</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>RH | Side | ASDVAv | RH | ASVzsVasdv</t>
+          <t>RH | Side | SDVBZ | RH | SDFBZFD</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -2182,12 +2182,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>RGSDG</t>
+          <t>SAvfas</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>DZSVBZDV</t>
+          <t>AFsDFFWAS</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>RH | Side | SDVBZ | RH | SDFBZFD</t>
+          <t>RH | Side | SFCc | RH | DVZDGV</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -2475,12 +2475,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SAvfas</t>
+          <t>VCNBVBN</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>AFsDFFWAS</t>
+          <t>VFBFCXB</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -2545,7 +2545,7 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>RH | Side | SFCc | RH | DVZDGV</t>
+          <t>RH | Side | FXBNXVB | RH | XBNDFXZBHDF</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -2768,12 +2768,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>VCNBVBN</t>
+          <t>CVDZV</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>VFBFCXB</t>
+          <t>ZCVDV</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -2838,7 +2838,7 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>RH | Side | FXBNXVB | RH | XBNDFXZBHDF</t>
+          <t>RH | Side | SDVd | RH | ZXVV</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -3061,12 +3061,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>CVDZV</t>
+          <t>VsgsdVDsvB</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>ZCVDV</t>
+          <t>DVasdvsdv</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -3354,7 +3354,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>VsgsdVDsvB</t>
+          <t>DASGVSDEGV</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -3647,12 +3647,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>DASGVSDEGV</t>
+          <t>sbghsdbghz</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>DVasdvsdv</t>
+          <t>sxDFBdzr</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -3717,7 +3717,7 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>RH | Side | SDVd | RH | ZXVV</t>
+          <t>RH | Side | sxzbdxf | RH | fndbzde</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -3940,12 +3940,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>sbghsdbghz</t>
+          <t>daGFAGD</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>sxDFBdzr</t>
+          <t>SDAGS</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -4233,12 +4233,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>daGFAGD</t>
+          <t>uiytrkiy</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>SDAGS</t>
+          <t>hglkclkhhl</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -4303,7 +4303,7 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>RH | Side | sxzbdxf | RH | fndbzde</t>
+          <t>RH | Side | ytidlk | RH | tdylkdl</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -4510,279 +4510,6 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="1" t="n">
-        <v>46323</v>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>FUSO Canter</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>FE84</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>uiytrkiy</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>hglkclkhhl</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>Weld Shop</t>
-        </is>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Over Tightening</t>
-        </is>
-      </c>
-      <c r="I13" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" t="n">
-        <v>1</v>
-      </c>
-      <c r="O13" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>RH | Side | ytidlk | RH | tdylkdl</t>
-        </is>
-      </c>
-      <c r="S13" t="inlineStr">
-        <is>
-          <t>Safety</t>
-        </is>
-      </c>
-      <c r="T13" t="inlineStr">
-        <is>
-          <t>Weld Shop</t>
-        </is>
-      </c>
-      <c r="U13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="V13" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="W13" t="n">
-        <v>1</v>
-      </c>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
-      <c r="AB13" t="inlineStr"/>
-      <c r="AC13" t="inlineStr"/>
-      <c r="AD13" t="inlineStr"/>
-      <c r="AE13" t="inlineStr"/>
-      <c r="AF13" t="inlineStr"/>
-      <c r="AG13" t="inlineStr"/>
-      <c r="AH13" t="inlineStr"/>
-      <c r="AI13" t="inlineStr"/>
-      <c r="AJ13" t="inlineStr"/>
-      <c r="AK13" t="inlineStr"/>
-      <c r="AL13" t="inlineStr"/>
-      <c r="AM13" t="inlineStr"/>
-      <c r="AN13" t="inlineStr"/>
-      <c r="AO13" t="inlineStr"/>
-      <c r="AP13" t="inlineStr"/>
-      <c r="AQ13" t="inlineStr"/>
-      <c r="AR13" t="inlineStr"/>
-      <c r="AS13" t="inlineStr"/>
-      <c r="AT13" t="inlineStr"/>
-      <c r="AU13" t="inlineStr"/>
-      <c r="AV13" t="inlineStr"/>
-      <c r="AW13" t="inlineStr"/>
-      <c r="AX13" t="inlineStr"/>
-      <c r="AY13" t="inlineStr"/>
-      <c r="AZ13" t="inlineStr"/>
-      <c r="BA13" t="inlineStr"/>
-      <c r="BB13" t="inlineStr"/>
-      <c r="BC13" t="inlineStr"/>
-      <c r="BD13" t="inlineStr"/>
-      <c r="BE13" t="inlineStr"/>
-      <c r="BF13" t="inlineStr"/>
-      <c r="BG13" t="inlineStr"/>
-      <c r="BH13" t="inlineStr"/>
-      <c r="BI13" t="inlineStr"/>
-      <c r="BJ13" t="inlineStr"/>
-      <c r="BK13" t="inlineStr"/>
-      <c r="BL13" t="inlineStr"/>
-      <c r="BM13" t="inlineStr"/>
-      <c r="BN13" t="inlineStr"/>
-      <c r="BO13" t="inlineStr"/>
-      <c r="BP13" t="inlineStr"/>
-      <c r="BQ13" t="inlineStr"/>
-      <c r="BR13" t="inlineStr"/>
-      <c r="BS13" t="inlineStr"/>
-      <c r="BT13" t="inlineStr"/>
-      <c r="BU13" t="inlineStr"/>
-      <c r="BV13" t="inlineStr"/>
-      <c r="BW13" t="inlineStr"/>
-      <c r="BX13" t="inlineStr"/>
-      <c r="BY13" t="inlineStr"/>
-      <c r="BZ13" t="inlineStr"/>
-      <c r="CA13" t="inlineStr"/>
-      <c r="CB13" t="inlineStr"/>
-      <c r="CC13" t="inlineStr"/>
-      <c r="CD13" t="inlineStr"/>
-      <c r="CE13" t="inlineStr"/>
-      <c r="CF13" t="inlineStr"/>
-      <c r="CG13" t="inlineStr"/>
-      <c r="CH13" t="inlineStr"/>
-      <c r="CI13" t="inlineStr"/>
-      <c r="CJ13" t="inlineStr"/>
-      <c r="CK13" t="inlineStr"/>
-      <c r="CL13" t="inlineStr"/>
-      <c r="CM13" t="inlineStr"/>
-      <c r="CN13" t="inlineStr"/>
-      <c r="CO13" t="inlineStr"/>
-      <c r="CP13" t="inlineStr"/>
-      <c r="CQ13" t="inlineStr"/>
-      <c r="CR13" t="inlineStr"/>
-      <c r="CS13" t="inlineStr"/>
-      <c r="CT13" t="inlineStr"/>
-      <c r="CU13" t="inlineStr"/>
-      <c r="CV13" t="inlineStr"/>
-      <c r="CW13" t="inlineStr"/>
-      <c r="CX13" t="inlineStr"/>
-      <c r="CY13" t="inlineStr"/>
-      <c r="CZ13" t="inlineStr"/>
-      <c r="DA13" t="inlineStr"/>
-      <c r="DB13" t="inlineStr"/>
-      <c r="DC13" t="inlineStr"/>
-      <c r="DD13" t="inlineStr"/>
-      <c r="DE13" t="inlineStr"/>
-      <c r="DF13" t="inlineStr"/>
-      <c r="DG13" t="inlineStr"/>
-      <c r="DH13" t="inlineStr"/>
-      <c r="DI13" t="inlineStr"/>
-      <c r="DJ13" t="inlineStr"/>
-      <c r="DK13" t="inlineStr"/>
-      <c r="DL13" t="inlineStr"/>
-      <c r="DM13" t="inlineStr"/>
-      <c r="DN13" t="inlineStr"/>
-      <c r="DO13" t="inlineStr"/>
-      <c r="DP13" t="inlineStr"/>
-      <c r="DQ13" t="inlineStr"/>
-      <c r="DR13" t="inlineStr"/>
-      <c r="DS13" t="inlineStr"/>
-      <c r="DT13" t="inlineStr"/>
-      <c r="DU13" t="inlineStr"/>
-      <c r="DV13" t="inlineStr"/>
-      <c r="DW13" t="inlineStr"/>
-      <c r="DX13" t="inlineStr"/>
-      <c r="DY13" t="inlineStr"/>
-      <c r="DZ13" t="inlineStr"/>
-      <c r="EA13" t="inlineStr"/>
-      <c r="EB13" t="inlineStr"/>
-      <c r="EC13" t="inlineStr"/>
-      <c r="ED13" t="inlineStr"/>
-      <c r="EE13" t="inlineStr"/>
-      <c r="EF13" t="inlineStr"/>
-      <c r="EG13" t="inlineStr"/>
-      <c r="EH13" t="inlineStr">
-        <is>
-          <t>Over Tightening</t>
-        </is>
-      </c>
-      <c r="EI13" t="inlineStr"/>
-      <c r="EJ13" t="inlineStr"/>
-      <c r="EK13" t="inlineStr"/>
-      <c r="EL13" t="inlineStr"/>
-      <c r="EM13" t="inlineStr"/>
-      <c r="EN13" t="inlineStr"/>
-      <c r="EO13" t="inlineStr"/>
-      <c r="EP13" t="inlineStr"/>
-      <c r="EQ13" t="inlineStr"/>
-      <c r="ER13" t="inlineStr"/>
-      <c r="ES13" t="inlineStr"/>
-      <c r="ET13" t="inlineStr"/>
-      <c r="EU13" t="inlineStr"/>
-      <c r="EV13" t="inlineStr"/>
-      <c r="EW13" t="inlineStr"/>
-      <c r="EX13" t="inlineStr"/>
-      <c r="EY13" t="inlineStr"/>
-      <c r="EZ13" t="inlineStr"/>
-      <c r="FA13" t="inlineStr"/>
-      <c r="FB13" t="inlineStr"/>
-      <c r="FC13" t="inlineStr"/>
-      <c r="FD13" t="inlineStr"/>
-      <c r="FE13" t="inlineStr"/>
-      <c r="FF13" t="inlineStr"/>
-      <c r="FG13" t="inlineStr"/>
-      <c r="FH13" t="inlineStr"/>
-      <c r="FI13" t="inlineStr"/>
-      <c r="FJ13" t="inlineStr"/>
-      <c r="FK13" t="inlineStr"/>
-      <c r="FL13" t="inlineStr">
-        <is>
-          <t>QFL4-20261028-0001</t>
-        </is>
-      </c>
-      <c r="FM13" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="FN13" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="FO13" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="FP13" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="FQ13" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>